<commit_message>
MT IMEA updater fix
</commit_message>
<xml_diff>
--- a/IMEA/harvest_prog_mt.xlsx
+++ b/IMEA/harvest_prog_mt.xlsx
@@ -839,8 +839,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -856,7 +864,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -864,12 +872,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1169,51 +1195,51 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:14">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:14">
-      <c r="A2" s="1">
+      <c r="A2" s="2">
         <v>45555</v>
       </c>
       <c r="B2" t="s">
@@ -1248,7 +1274,7 @@
       </c>
     </row>
     <row r="3" spans="1:14">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>45555</v>
       </c>
       <c r="B3" t="s">
@@ -1289,7 +1315,7 @@
       </c>
     </row>
     <row r="4" spans="1:14">
-      <c r="A4" s="1">
+      <c r="A4" s="2">
         <v>45555</v>
       </c>
       <c r="B4" t="s">
@@ -1330,7 +1356,7 @@
       </c>
     </row>
     <row r="5" spans="1:14">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>45555</v>
       </c>
       <c r="B5" t="s">
@@ -1371,7 +1397,7 @@
       </c>
     </row>
     <row r="6" spans="1:14">
-      <c r="A6" s="1">
+      <c r="A6" s="2">
         <v>45555</v>
       </c>
       <c r="B6" t="s">
@@ -1412,7 +1438,7 @@
       </c>
     </row>
     <row r="7" spans="1:14">
-      <c r="A7" s="1">
+      <c r="A7" s="2">
         <v>45555</v>
       </c>
       <c r="B7" t="s">
@@ -1453,7 +1479,7 @@
       </c>
     </row>
     <row r="8" spans="1:14">
-      <c r="A8" s="1">
+      <c r="A8" s="2">
         <v>45555</v>
       </c>
       <c r="B8" t="s">
@@ -1494,7 +1520,7 @@
       </c>
     </row>
     <row r="9" spans="1:14">
-      <c r="A9" s="1">
+      <c r="A9" s="2">
         <v>45555</v>
       </c>
       <c r="B9" t="s">
@@ -1535,7 +1561,7 @@
       </c>
     </row>
     <row r="10" spans="1:14">
-      <c r="A10" s="1">
+      <c r="A10" s="2">
         <v>45835</v>
       </c>
       <c r="B10" t="s">
@@ -1570,7 +1596,7 @@
       </c>
     </row>
     <row r="11" spans="1:14">
-      <c r="A11" s="1">
+      <c r="A11" s="2">
         <v>45835</v>
       </c>
       <c r="B11" t="s">
@@ -1611,7 +1637,7 @@
       </c>
     </row>
     <row r="12" spans="1:14">
-      <c r="A12" s="1">
+      <c r="A12" s="2">
         <v>45835</v>
       </c>
       <c r="B12" t="s">
@@ -1652,7 +1678,7 @@
       </c>
     </row>
     <row r="13" spans="1:14">
-      <c r="A13" s="1">
+      <c r="A13" s="2">
         <v>45835</v>
       </c>
       <c r="B13" t="s">
@@ -1693,7 +1719,7 @@
       </c>
     </row>
     <row r="14" spans="1:14">
-      <c r="A14" s="1">
+      <c r="A14" s="2">
         <v>45835</v>
       </c>
       <c r="B14" t="s">
@@ -1734,7 +1760,7 @@
       </c>
     </row>
     <row r="15" spans="1:14">
-      <c r="A15" s="1">
+      <c r="A15" s="2">
         <v>45835</v>
       </c>
       <c r="B15" t="s">
@@ -1775,7 +1801,7 @@
       </c>
     </row>
     <row r="16" spans="1:14">
-      <c r="A16" s="1">
+      <c r="A16" s="2">
         <v>45835</v>
       </c>
       <c r="B16" t="s">
@@ -1816,7 +1842,7 @@
       </c>
     </row>
     <row r="17" spans="1:14">
-      <c r="A17" s="1">
+      <c r="A17" s="2">
         <v>45835</v>
       </c>
       <c r="B17" t="s">
@@ -1857,7 +1883,7 @@
       </c>
     </row>
     <row r="18" spans="1:14">
-      <c r="A18" s="1">
+      <c r="A18" s="2">
         <v>45842</v>
       </c>
       <c r="B18" t="s">
@@ -1895,7 +1921,7 @@
       </c>
     </row>
     <row r="19" spans="1:14">
-      <c r="A19" s="1">
+      <c r="A19" s="2">
         <v>45842</v>
       </c>
       <c r="B19" t="s">
@@ -1936,7 +1962,7 @@
       </c>
     </row>
     <row r="20" spans="1:14">
-      <c r="A20" s="1">
+      <c r="A20" s="2">
         <v>45842</v>
       </c>
       <c r="B20" t="s">
@@ -1980,7 +2006,7 @@
       </c>
     </row>
     <row r="21" spans="1:14">
-      <c r="A21" s="1">
+      <c r="A21" s="2">
         <v>45842</v>
       </c>
       <c r="B21" t="s">
@@ -2024,7 +2050,7 @@
       </c>
     </row>
     <row r="22" spans="1:14">
-      <c r="A22" s="1">
+      <c r="A22" s="2">
         <v>45842</v>
       </c>
       <c r="B22" t="s">
@@ -2065,7 +2091,7 @@
       </c>
     </row>
     <row r="23" spans="1:14">
-      <c r="A23" s="1">
+      <c r="A23" s="2">
         <v>45842</v>
       </c>
       <c r="B23" t="s">
@@ -2106,7 +2132,7 @@
       </c>
     </row>
     <row r="24" spans="1:14">
-      <c r="A24" s="1">
+      <c r="A24" s="2">
         <v>45842</v>
       </c>
       <c r="B24" t="s">
@@ -2147,7 +2173,7 @@
       </c>
     </row>
     <row r="25" spans="1:14">
-      <c r="A25" s="1">
+      <c r="A25" s="2">
         <v>45842</v>
       </c>
       <c r="B25" t="s">
@@ -2191,7 +2217,7 @@
       </c>
     </row>
     <row r="26" spans="1:14">
-      <c r="A26" s="1">
+      <c r="A26" s="2">
         <v>45849</v>
       </c>
       <c r="B26" t="s">
@@ -2229,7 +2255,7 @@
       </c>
     </row>
     <row r="27" spans="1:14">
-      <c r="A27" s="1">
+      <c r="A27" s="2">
         <v>45849</v>
       </c>
       <c r="B27" t="s">
@@ -2273,7 +2299,7 @@
       </c>
     </row>
     <row r="28" spans="1:14">
-      <c r="A28" s="1">
+      <c r="A28" s="2">
         <v>45849</v>
       </c>
       <c r="B28" t="s">
@@ -2317,7 +2343,7 @@
       </c>
     </row>
     <row r="29" spans="1:14">
-      <c r="A29" s="1">
+      <c r="A29" s="2">
         <v>45849</v>
       </c>
       <c r="B29" t="s">
@@ -2361,7 +2387,7 @@
       </c>
     </row>
     <row r="30" spans="1:14">
-      <c r="A30" s="1">
+      <c r="A30" s="2">
         <v>45849</v>
       </c>
       <c r="B30" t="s">
@@ -2402,7 +2428,7 @@
       </c>
     </row>
     <row r="31" spans="1:14">
-      <c r="A31" s="1">
+      <c r="A31" s="2">
         <v>45849</v>
       </c>
       <c r="B31" t="s">
@@ -2443,7 +2469,7 @@
       </c>
     </row>
     <row r="32" spans="1:14">
-      <c r="A32" s="1">
+      <c r="A32" s="2">
         <v>45849</v>
       </c>
       <c r="B32" t="s">
@@ -2487,7 +2513,7 @@
       </c>
     </row>
     <row r="33" spans="1:14">
-      <c r="A33" s="1">
+      <c r="A33" s="2">
         <v>45849</v>
       </c>
       <c r="B33" t="s">
@@ -2531,7 +2557,7 @@
       </c>
     </row>
     <row r="34" spans="1:14">
-      <c r="A34" s="1">
+      <c r="A34" s="2">
         <v>45856</v>
       </c>
       <c r="B34" t="s">
@@ -2569,7 +2595,7 @@
       </c>
     </row>
     <row r="35" spans="1:14">
-      <c r="A35" s="1">
+      <c r="A35" s="2">
         <v>45856</v>
       </c>
       <c r="B35" t="s">
@@ -2613,7 +2639,7 @@
       </c>
     </row>
     <row r="36" spans="1:14">
-      <c r="A36" s="1">
+      <c r="A36" s="2">
         <v>45856</v>
       </c>
       <c r="B36" t="s">
@@ -2657,7 +2683,7 @@
       </c>
     </row>
     <row r="37" spans="1:14">
-      <c r="A37" s="1">
+      <c r="A37" s="2">
         <v>45856</v>
       </c>
       <c r="B37" t="s">
@@ -2701,7 +2727,7 @@
       </c>
     </row>
     <row r="38" spans="1:14">
-      <c r="A38" s="1">
+      <c r="A38" s="2">
         <v>45856</v>
       </c>
       <c r="B38" t="s">
@@ -2745,7 +2771,7 @@
       </c>
     </row>
     <row r="39" spans="1:14">
-      <c r="A39" s="1">
+      <c r="A39" s="2">
         <v>45856</v>
       </c>
       <c r="B39" t="s">
@@ -2786,7 +2812,7 @@
       </c>
     </row>
     <row r="40" spans="1:14">
-      <c r="A40" s="1">
+      <c r="A40" s="2">
         <v>45856</v>
       </c>
       <c r="B40" t="s">
@@ -2830,7 +2856,7 @@
       </c>
     </row>
     <row r="41" spans="1:14">
-      <c r="A41" s="1">
+      <c r="A41" s="2">
         <v>45856</v>
       </c>
       <c r="B41" t="s">
@@ -2874,7 +2900,7 @@
       </c>
     </row>
     <row r="42" spans="1:14">
-      <c r="A42" s="1">
+      <c r="A42" s="2">
         <v>45863</v>
       </c>
       <c r="B42" t="s">
@@ -2912,7 +2938,7 @@
       </c>
     </row>
     <row r="43" spans="1:14">
-      <c r="A43" s="1">
+      <c r="A43" s="2">
         <v>45863</v>
       </c>
       <c r="B43" t="s">
@@ -2956,7 +2982,7 @@
       </c>
     </row>
     <row r="44" spans="1:14">
-      <c r="A44" s="1">
+      <c r="A44" s="2">
         <v>45863</v>
       </c>
       <c r="B44" t="s">
@@ -3000,7 +3026,7 @@
       </c>
     </row>
     <row r="45" spans="1:14">
-      <c r="A45" s="1">
+      <c r="A45" s="2">
         <v>45863</v>
       </c>
       <c r="B45" t="s">
@@ -3044,7 +3070,7 @@
       </c>
     </row>
     <row r="46" spans="1:14">
-      <c r="A46" s="1">
+      <c r="A46" s="2">
         <v>45863</v>
       </c>
       <c r="B46" t="s">
@@ -3088,7 +3114,7 @@
       </c>
     </row>
     <row r="47" spans="1:14">
-      <c r="A47" s="1">
+      <c r="A47" s="2">
         <v>45863</v>
       </c>
       <c r="B47" t="s">
@@ -3129,7 +3155,7 @@
       </c>
     </row>
     <row r="48" spans="1:14">
-      <c r="A48" s="1">
+      <c r="A48" s="2">
         <v>45863</v>
       </c>
       <c r="B48" t="s">
@@ -3173,7 +3199,7 @@
       </c>
     </row>
     <row r="49" spans="1:14">
-      <c r="A49" s="1">
+      <c r="A49" s="2">
         <v>45863</v>
       </c>
       <c r="B49" t="s">
@@ -3217,7 +3243,7 @@
       </c>
     </row>
     <row r="50" spans="1:14">
-      <c r="A50" s="1">
+      <c r="A50" s="2">
         <v>45870</v>
       </c>
       <c r="B50" t="s">
@@ -3255,7 +3281,7 @@
       </c>
     </row>
     <row r="51" spans="1:14">
-      <c r="A51" s="1">
+      <c r="A51" s="2">
         <v>45870</v>
       </c>
       <c r="B51" t="s">
@@ -3299,7 +3325,7 @@
       </c>
     </row>
     <row r="52" spans="1:14">
-      <c r="A52" s="1">
+      <c r="A52" s="2">
         <v>45870</v>
       </c>
       <c r="B52" t="s">
@@ -3343,7 +3369,7 @@
       </c>
     </row>
     <row r="53" spans="1:14">
-      <c r="A53" s="1">
+      <c r="A53" s="2">
         <v>45870</v>
       </c>
       <c r="B53" t="s">
@@ -3387,7 +3413,7 @@
       </c>
     </row>
     <row r="54" spans="1:14">
-      <c r="A54" s="1">
+      <c r="A54" s="2">
         <v>45870</v>
       </c>
       <c r="B54" t="s">
@@ -3431,7 +3457,7 @@
       </c>
     </row>
     <row r="55" spans="1:14">
-      <c r="A55" s="1">
+      <c r="A55" s="2">
         <v>45870</v>
       </c>
       <c r="B55" t="s">
@@ -3472,7 +3498,7 @@
       </c>
     </row>
     <row r="56" spans="1:14">
-      <c r="A56" s="1">
+      <c r="A56" s="2">
         <v>45870</v>
       </c>
       <c r="B56" t="s">
@@ -3516,7 +3542,7 @@
       </c>
     </row>
     <row r="57" spans="1:14">
-      <c r="A57" s="1">
+      <c r="A57" s="2">
         <v>45870</v>
       </c>
       <c r="B57" t="s">
@@ -3560,7 +3586,7 @@
       </c>
     </row>
     <row r="58" spans="1:14">
-      <c r="A58" s="1">
+      <c r="A58" s="2">
         <v>45877</v>
       </c>
       <c r="B58" t="s">
@@ -3598,7 +3624,7 @@
       </c>
     </row>
     <row r="59" spans="1:14">
-      <c r="A59" s="1">
+      <c r="A59" s="2">
         <v>45877</v>
       </c>
       <c r="B59" t="s">
@@ -3642,7 +3668,7 @@
       </c>
     </row>
     <row r="60" spans="1:14">
-      <c r="A60" s="1">
+      <c r="A60" s="2">
         <v>45877</v>
       </c>
       <c r="B60" t="s">
@@ -3686,7 +3712,7 @@
       </c>
     </row>
     <row r="61" spans="1:14">
-      <c r="A61" s="1">
+      <c r="A61" s="2">
         <v>45877</v>
       </c>
       <c r="B61" t="s">
@@ -3730,7 +3756,7 @@
       </c>
     </row>
     <row r="62" spans="1:14">
-      <c r="A62" s="1">
+      <c r="A62" s="2">
         <v>45877</v>
       </c>
       <c r="B62" t="s">
@@ -3774,7 +3800,7 @@
       </c>
     </row>
     <row r="63" spans="1:14">
-      <c r="A63" s="1">
+      <c r="A63" s="2">
         <v>45877</v>
       </c>
       <c r="B63" t="s">
@@ -3815,7 +3841,7 @@
       </c>
     </row>
     <row r="64" spans="1:14">
-      <c r="A64" s="1">
+      <c r="A64" s="2">
         <v>45877</v>
       </c>
       <c r="B64" t="s">
@@ -3859,7 +3885,7 @@
       </c>
     </row>
     <row r="65" spans="1:14">
-      <c r="A65" s="1">
+      <c r="A65" s="2">
         <v>45877</v>
       </c>
       <c r="B65" t="s">
@@ -3903,7 +3929,7 @@
       </c>
     </row>
     <row r="66" spans="1:14">
-      <c r="A66" s="1">
+      <c r="A66" s="2">
         <v>45884</v>
       </c>
       <c r="B66" t="s">
@@ -3941,7 +3967,7 @@
       </c>
     </row>
     <row r="67" spans="1:14">
-      <c r="A67" s="1">
+      <c r="A67" s="2">
         <v>45884</v>
       </c>
       <c r="B67" t="s">
@@ -3985,7 +4011,7 @@
       </c>
     </row>
     <row r="68" spans="1:14">
-      <c r="A68" s="1">
+      <c r="A68" s="2">
         <v>45884</v>
       </c>
       <c r="B68" t="s">
@@ -4029,7 +4055,7 @@
       </c>
     </row>
     <row r="69" spans="1:14">
-      <c r="A69" s="1">
+      <c r="A69" s="2">
         <v>45884</v>
       </c>
       <c r="B69" t="s">
@@ -4073,7 +4099,7 @@
       </c>
     </row>
     <row r="70" spans="1:14">
-      <c r="A70" s="1">
+      <c r="A70" s="2">
         <v>45884</v>
       </c>
       <c r="B70" t="s">
@@ -4117,7 +4143,7 @@
       </c>
     </row>
     <row r="71" spans="1:14">
-      <c r="A71" s="1">
+      <c r="A71" s="2">
         <v>45884</v>
       </c>
       <c r="B71" t="s">
@@ -4158,7 +4184,7 @@
       </c>
     </row>
     <row r="72" spans="1:14">
-      <c r="A72" s="1">
+      <c r="A72" s="2">
         <v>45884</v>
       </c>
       <c r="B72" t="s">
@@ -4202,7 +4228,7 @@
       </c>
     </row>
     <row r="73" spans="1:14">
-      <c r="A73" s="1">
+      <c r="A73" s="2">
         <v>45884</v>
       </c>
       <c r="B73" t="s">
@@ -4246,7 +4272,7 @@
       </c>
     </row>
     <row r="74" spans="1:14">
-      <c r="A74" s="1">
+      <c r="A74" s="2">
         <v>45891</v>
       </c>
       <c r="B74" t="s">
@@ -4284,7 +4310,7 @@
       </c>
     </row>
     <row r="75" spans="1:14">
-      <c r="A75" s="1">
+      <c r="A75" s="2">
         <v>45891</v>
       </c>
       <c r="B75" t="s">
@@ -4328,7 +4354,7 @@
       </c>
     </row>
     <row r="76" spans="1:14">
-      <c r="A76" s="1">
+      <c r="A76" s="2">
         <v>45891</v>
       </c>
       <c r="B76" t="s">
@@ -4372,7 +4398,7 @@
       </c>
     </row>
     <row r="77" spans="1:14">
-      <c r="A77" s="1">
+      <c r="A77" s="2">
         <v>45891</v>
       </c>
       <c r="B77" t="s">
@@ -4416,7 +4442,7 @@
       </c>
     </row>
     <row r="78" spans="1:14">
-      <c r="A78" s="1">
+      <c r="A78" s="2">
         <v>45891</v>
       </c>
       <c r="B78" t="s">
@@ -4460,7 +4486,7 @@
       </c>
     </row>
     <row r="79" spans="1:14">
-      <c r="A79" s="1">
+      <c r="A79" s="2">
         <v>45891</v>
       </c>
       <c r="B79" t="s">
@@ -4501,7 +4527,7 @@
       </c>
     </row>
     <row r="80" spans="1:14">
-      <c r="A80" s="1">
+      <c r="A80" s="2">
         <v>45891</v>
       </c>
       <c r="B80" t="s">
@@ -4545,7 +4571,7 @@
       </c>
     </row>
     <row r="81" spans="1:14">
-      <c r="A81" s="1">
+      <c r="A81" s="2">
         <v>45891</v>
       </c>
       <c r="B81" t="s">
@@ -4589,7 +4615,7 @@
       </c>
     </row>
     <row r="82" spans="1:14">
-      <c r="A82" s="1">
+      <c r="A82" s="2">
         <v>45898</v>
       </c>
       <c r="B82" t="s">
@@ -4627,7 +4653,7 @@
       </c>
     </row>
     <row r="83" spans="1:14">
-      <c r="A83" s="1">
+      <c r="A83" s="2">
         <v>45898</v>
       </c>
       <c r="B83" t="s">
@@ -4671,7 +4697,7 @@
       </c>
     </row>
     <row r="84" spans="1:14">
-      <c r="A84" s="1">
+      <c r="A84" s="2">
         <v>45898</v>
       </c>
       <c r="B84" t="s">
@@ -4715,7 +4741,7 @@
       </c>
     </row>
     <row r="85" spans="1:14">
-      <c r="A85" s="1">
+      <c r="A85" s="2">
         <v>45898</v>
       </c>
       <c r="B85" t="s">
@@ -4759,7 +4785,7 @@
       </c>
     </row>
     <row r="86" spans="1:14">
-      <c r="A86" s="1">
+      <c r="A86" s="2">
         <v>45898</v>
       </c>
       <c r="B86" t="s">
@@ -4803,7 +4829,7 @@
       </c>
     </row>
     <row r="87" spans="1:14">
-      <c r="A87" s="1">
+      <c r="A87" s="2">
         <v>45898</v>
       </c>
       <c r="B87" t="s">
@@ -4844,7 +4870,7 @@
       </c>
     </row>
     <row r="88" spans="1:14">
-      <c r="A88" s="1">
+      <c r="A88" s="2">
         <v>45898</v>
       </c>
       <c r="B88" t="s">
@@ -4888,7 +4914,7 @@
       </c>
     </row>
     <row r="89" spans="1:14">
-      <c r="A89" s="1">
+      <c r="A89" s="2">
         <v>45898</v>
       </c>
       <c r="B89" t="s">
@@ -4932,7 +4958,7 @@
       </c>
     </row>
     <row r="90" spans="1:14">
-      <c r="A90" s="1">
+      <c r="A90" s="2">
         <v>45905</v>
       </c>
       <c r="B90" t="s">
@@ -4970,7 +4996,7 @@
       </c>
     </row>
     <row r="91" spans="1:14">
-      <c r="A91" s="1">
+      <c r="A91" s="2">
         <v>45905</v>
       </c>
       <c r="B91" t="s">
@@ -5014,7 +5040,7 @@
       </c>
     </row>
     <row r="92" spans="1:14">
-      <c r="A92" s="1">
+      <c r="A92" s="2">
         <v>45905</v>
       </c>
       <c r="B92" t="s">
@@ -5058,7 +5084,7 @@
       </c>
     </row>
     <row r="93" spans="1:14">
-      <c r="A93" s="1">
+      <c r="A93" s="2">
         <v>45905</v>
       </c>
       <c r="B93" t="s">
@@ -5102,7 +5128,7 @@
       </c>
     </row>
     <row r="94" spans="1:14">
-      <c r="A94" s="1">
+      <c r="A94" s="2">
         <v>45905</v>
       </c>
       <c r="B94" t="s">
@@ -5146,7 +5172,7 @@
       </c>
     </row>
     <row r="95" spans="1:14">
-      <c r="A95" s="1">
+      <c r="A95" s="2">
         <v>45905</v>
       </c>
       <c r="B95" t="s">
@@ -5187,7 +5213,7 @@
       </c>
     </row>
     <row r="96" spans="1:14">
-      <c r="A96" s="1">
+      <c r="A96" s="2">
         <v>45905</v>
       </c>
       <c r="B96" t="s">
@@ -5231,7 +5257,7 @@
       </c>
     </row>
     <row r="97" spans="1:14">
-      <c r="A97" s="1">
+      <c r="A97" s="2">
         <v>45905</v>
       </c>
       <c r="B97" t="s">
@@ -5275,7 +5301,7 @@
       </c>
     </row>
     <row r="98" spans="1:14">
-      <c r="A98" s="1">
+      <c r="A98" s="2">
         <v>45912</v>
       </c>
       <c r="B98" t="s">
@@ -5313,7 +5339,7 @@
       </c>
     </row>
     <row r="99" spans="1:14">
-      <c r="A99" s="1">
+      <c r="A99" s="2">
         <v>45912</v>
       </c>
       <c r="B99" t="s">
@@ -5357,7 +5383,7 @@
       </c>
     </row>
     <row r="100" spans="1:14">
-      <c r="A100" s="1">
+      <c r="A100" s="2">
         <v>45912</v>
       </c>
       <c r="B100" t="s">
@@ -5401,7 +5427,7 @@
       </c>
     </row>
     <row r="101" spans="1:14">
-      <c r="A101" s="1">
+      <c r="A101" s="2">
         <v>45912</v>
       </c>
       <c r="B101" t="s">
@@ -5445,7 +5471,7 @@
       </c>
     </row>
     <row r="102" spans="1:14">
-      <c r="A102" s="1">
+      <c r="A102" s="2">
         <v>45912</v>
       </c>
       <c r="B102" t="s">
@@ -5489,7 +5515,7 @@
       </c>
     </row>
     <row r="103" spans="1:14">
-      <c r="A103" s="1">
+      <c r="A103" s="2">
         <v>45912</v>
       </c>
       <c r="B103" t="s">
@@ -5530,7 +5556,7 @@
       </c>
     </row>
     <row r="104" spans="1:14">
-      <c r="A104" s="1">
+      <c r="A104" s="2">
         <v>45912</v>
       </c>
       <c r="B104" t="s">
@@ -5574,7 +5600,7 @@
       </c>
     </row>
     <row r="105" spans="1:14">
-      <c r="A105" s="1">
+      <c r="A105" s="2">
         <v>45912</v>
       </c>
       <c r="B105" t="s">
@@ -5618,7 +5644,7 @@
       </c>
     </row>
     <row r="106" spans="1:14">
-      <c r="A106" s="1">
+      <c r="A106" s="2">
         <v>45919</v>
       </c>
       <c r="B106" t="s">
@@ -5656,7 +5682,7 @@
       </c>
     </row>
     <row r="107" spans="1:14">
-      <c r="A107" s="1">
+      <c r="A107" s="2">
         <v>45919</v>
       </c>
       <c r="B107" t="s">
@@ -5700,7 +5726,7 @@
       </c>
     </row>
     <row r="108" spans="1:14">
-      <c r="A108" s="1">
+      <c r="A108" s="2">
         <v>45919</v>
       </c>
       <c r="B108" t="s">
@@ -5744,7 +5770,7 @@
       </c>
     </row>
     <row r="109" spans="1:14">
-      <c r="A109" s="1">
+      <c r="A109" s="2">
         <v>45919</v>
       </c>
       <c r="B109" t="s">
@@ -5788,7 +5814,7 @@
       </c>
     </row>
     <row r="110" spans="1:14">
-      <c r="A110" s="1">
+      <c r="A110" s="2">
         <v>45919</v>
       </c>
       <c r="B110" t="s">
@@ -5832,7 +5858,7 @@
       </c>
     </row>
     <row r="111" spans="1:14">
-      <c r="A111" s="1">
+      <c r="A111" s="2">
         <v>45919</v>
       </c>
       <c r="B111" t="s">
@@ -5873,7 +5899,7 @@
       </c>
     </row>
     <row r="112" spans="1:14">
-      <c r="A112" s="1">
+      <c r="A112" s="2">
         <v>45919</v>
       </c>
       <c r="B112" t="s">
@@ -5917,7 +5943,7 @@
       </c>
     </row>
     <row r="113" spans="1:14">
-      <c r="A113" s="1">
+      <c r="A113" s="2">
         <v>45919</v>
       </c>
       <c r="B113" t="s">
@@ -5961,7 +5987,7 @@
       </c>
     </row>
     <row r="114" spans="1:14">
-      <c r="A114" s="1">
+      <c r="A114" s="2">
         <v>45926</v>
       </c>
       <c r="B114" t="s">
@@ -5999,7 +6025,7 @@
       </c>
     </row>
     <row r="115" spans="1:14">
-      <c r="A115" s="1">
+      <c r="A115" s="2">
         <v>45926</v>
       </c>
       <c r="B115" t="s">
@@ -6043,7 +6069,7 @@
       </c>
     </row>
     <row r="116" spans="1:14">
-      <c r="A116" s="1">
+      <c r="A116" s="2">
         <v>45926</v>
       </c>
       <c r="B116" t="s">
@@ -6087,7 +6113,7 @@
       </c>
     </row>
     <row r="117" spans="1:14">
-      <c r="A117" s="1">
+      <c r="A117" s="2">
         <v>45926</v>
       </c>
       <c r="B117" t="s">
@@ -6131,7 +6157,7 @@
       </c>
     </row>
     <row r="118" spans="1:14">
-      <c r="A118" s="1">
+      <c r="A118" s="2">
         <v>45926</v>
       </c>
       <c r="B118" t="s">
@@ -6175,7 +6201,7 @@
       </c>
     </row>
     <row r="119" spans="1:14">
-      <c r="A119" s="1">
+      <c r="A119" s="2">
         <v>45926</v>
       </c>
       <c r="B119" t="s">
@@ -6216,7 +6242,7 @@
       </c>
     </row>
     <row r="120" spans="1:14">
-      <c r="A120" s="1">
+      <c r="A120" s="2">
         <v>45926</v>
       </c>
       <c r="B120" t="s">
@@ -6260,7 +6286,7 @@
       </c>
     </row>
     <row r="121" spans="1:14">
-      <c r="A121" s="1">
+      <c r="A121" s="2">
         <v>45926</v>
       </c>
       <c r="B121" t="s">
@@ -6314,39 +6340,39 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:10">
-      <c r="A2" s="1">
+      <c r="A2" s="2">
         <v>45555</v>
       </c>
       <c r="B2" t="s">
@@ -6378,7 +6404,7 @@
       </c>
     </row>
     <row r="3" spans="1:10">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>45835</v>
       </c>
       <c r="B3" t="s">
@@ -6410,7 +6436,7 @@
       </c>
     </row>
     <row r="4" spans="1:10">
-      <c r="A4" s="1">
+      <c r="A4" s="2">
         <v>45842</v>
       </c>
       <c r="B4" t="s">
@@ -6442,7 +6468,7 @@
       </c>
     </row>
     <row r="5" spans="1:10">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>45849</v>
       </c>
       <c r="B5" t="s">
@@ -6474,7 +6500,7 @@
       </c>
     </row>
     <row r="6" spans="1:10">
-      <c r="A6" s="1">
+      <c r="A6" s="2">
         <v>45856</v>
       </c>
       <c r="B6" t="s">
@@ -6506,7 +6532,7 @@
       </c>
     </row>
     <row r="7" spans="1:10">
-      <c r="A7" s="1">
+      <c r="A7" s="2">
         <v>45863</v>
       </c>
       <c r="B7" t="s">
@@ -6538,7 +6564,7 @@
       </c>
     </row>
     <row r="8" spans="1:10">
-      <c r="A8" s="1">
+      <c r="A8" s="2">
         <v>45870</v>
       </c>
       <c r="B8" t="s">
@@ -6570,7 +6596,7 @@
       </c>
     </row>
     <row r="9" spans="1:10">
-      <c r="A9" s="1">
+      <c r="A9" s="2">
         <v>45877</v>
       </c>
       <c r="B9" t="s">
@@ -6602,7 +6628,7 @@
       </c>
     </row>
     <row r="10" spans="1:10">
-      <c r="A10" s="1">
+      <c r="A10" s="2">
         <v>45884</v>
       </c>
       <c r="B10" t="s">
@@ -6634,7 +6660,7 @@
       </c>
     </row>
     <row r="11" spans="1:10">
-      <c r="A11" s="1">
+      <c r="A11" s="2">
         <v>45891</v>
       </c>
       <c r="B11" t="s">
@@ -6666,7 +6692,7 @@
       </c>
     </row>
     <row r="12" spans="1:10">
-      <c r="A12" s="1">
+      <c r="A12" s="2">
         <v>45898</v>
       </c>
       <c r="B12" t="s">
@@ -6698,7 +6724,7 @@
       </c>
     </row>
     <row r="13" spans="1:10">
-      <c r="A13" s="1">
+      <c r="A13" s="2">
         <v>45905</v>
       </c>
       <c r="B13" t="s">
@@ -6730,7 +6756,7 @@
       </c>
     </row>
     <row r="14" spans="1:10">
-      <c r="A14" s="1">
+      <c r="A14" s="2">
         <v>45912</v>
       </c>
       <c r="B14" t="s">
@@ -6762,7 +6788,7 @@
       </c>
     </row>
     <row r="15" spans="1:10">
-      <c r="A15" s="1">
+      <c r="A15" s="2">
         <v>45919</v>
       </c>
       <c r="B15" t="s">
@@ -6794,7 +6820,7 @@
       </c>
     </row>
     <row r="16" spans="1:10">
-      <c r="A16" s="1">
+      <c r="A16" s="2">
         <v>45926</v>
       </c>
       <c r="B16" t="s">
@@ -6836,13 +6862,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>47</v>
       </c>
     </row>
@@ -6850,7 +6876,7 @@
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="1">
+      <c r="B2" s="2">
         <v>45555</v>
       </c>
       <c r="C2">
@@ -6861,7 +6887,7 @@
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B3" s="2">
         <v>45835</v>
       </c>
       <c r="C3">
@@ -6872,7 +6898,7 @@
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B4" s="2">
         <v>45842</v>
       </c>
       <c r="C4">
@@ -6883,7 +6909,7 @@
       <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" s="1">
+      <c r="B5" s="2">
         <v>45849</v>
       </c>
       <c r="C5">
@@ -6894,7 +6920,7 @@
       <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6" s="1">
+      <c r="B6" s="2">
         <v>45856</v>
       </c>
       <c r="C6">
@@ -6905,7 +6931,7 @@
       <c r="A7">
         <v>6</v>
       </c>
-      <c r="B7" s="1">
+      <c r="B7" s="2">
         <v>45863</v>
       </c>
       <c r="C7">
@@ -6916,7 +6942,7 @@
       <c r="A8">
         <v>7</v>
       </c>
-      <c r="B8" s="1">
+      <c r="B8" s="2">
         <v>45870</v>
       </c>
       <c r="C8">
@@ -6927,7 +6953,7 @@
       <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9" s="1">
+      <c r="B9" s="2">
         <v>45877</v>
       </c>
       <c r="C9">
@@ -6938,7 +6964,7 @@
       <c r="A10">
         <v>9</v>
       </c>
-      <c r="B10" s="1">
+      <c r="B10" s="2">
         <v>45884</v>
       </c>
       <c r="C10">
@@ -6949,7 +6975,7 @@
       <c r="A11">
         <v>10</v>
       </c>
-      <c r="B11" s="1">
+      <c r="B11" s="2">
         <v>45891</v>
       </c>
       <c r="C11">
@@ -6960,7 +6986,7 @@
       <c r="A12">
         <v>11</v>
       </c>
-      <c r="B12" s="1">
+      <c r="B12" s="2">
         <v>45898</v>
       </c>
       <c r="C12">
@@ -6971,7 +6997,7 @@
       <c r="A13">
         <v>12</v>
       </c>
-      <c r="B13" s="1">
+      <c r="B13" s="2">
         <v>45905</v>
       </c>
       <c r="C13">
@@ -6982,7 +7008,7 @@
       <c r="A14">
         <v>13</v>
       </c>
-      <c r="B14" s="1">
+      <c r="B14" s="2">
         <v>45912</v>
       </c>
       <c r="C14">
@@ -6993,7 +7019,7 @@
       <c r="A15">
         <v>14</v>
       </c>
-      <c r="B15" s="1">
+      <c r="B15" s="2">
         <v>45919</v>
       </c>
       <c r="C15">
@@ -7004,7 +7030,7 @@
       <c r="A16">
         <v>15</v>
       </c>
-      <c r="B16" s="1">
+      <c r="B16" s="2">
         <v>45926</v>
       </c>
       <c r="C16">
@@ -7022,196 +7048,196 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:64">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AF1" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AG1" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AH1" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="AI1" t="s">
+      <c r="AI1" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="AJ1" t="s">
+      <c r="AJ1" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="AK1" t="s">
+      <c r="AK1" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="AL1" t="s">
+      <c r="AL1" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="AM1" t="s">
+      <c r="AM1" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="AN1" t="s">
+      <c r="AN1" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="AO1" t="s">
+      <c r="AO1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="AP1" t="s">
+      <c r="AP1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="AQ1" t="s">
+      <c r="AQ1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="AR1" t="s">
+      <c r="AR1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="AS1" t="s">
+      <c r="AS1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="AT1" t="s">
+      <c r="AT1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="AU1" t="s">
+      <c r="AU1" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="AV1" t="s">
+      <c r="AV1" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="AW1" t="s">
+      <c r="AW1" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="AX1" t="s">
+      <c r="AX1" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="AY1" t="s">
+      <c r="AY1" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="AZ1" t="s">
+      <c r="AZ1" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="BA1" t="s">
+      <c r="BA1" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="BB1" t="s">
+      <c r="BB1" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="BC1" t="s">
+      <c r="BC1" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="BD1" t="s">
+      <c r="BD1" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="BE1" t="s">
+      <c r="BE1" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="BF1" t="s">
+      <c r="BF1" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="BG1" t="s">
+      <c r="BG1" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="BH1" t="s">
+      <c r="BH1" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="BI1" t="s">
+      <c r="BI1" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="BJ1" t="s">
+      <c r="BJ1" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="BK1" t="s">
+      <c r="BK1" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="BL1" t="s">
+      <c r="BL1" s="1" t="s">
         <v>111</v>
       </c>
     </row>
@@ -7315,7 +7341,7 @@
       <c r="AY2" t="s">
         <v>20</v>
       </c>
-      <c r="AZ2" s="1">
+      <c r="AZ2" s="2">
         <v>45555</v>
       </c>
       <c r="BA2" t="s">
@@ -7434,7 +7460,7 @@
       <c r="AY3" t="s">
         <v>21</v>
       </c>
-      <c r="AZ3" s="1">
+      <c r="AZ3" s="2">
         <v>45555</v>
       </c>
       <c r="BA3" t="s">
@@ -7553,7 +7579,7 @@
       <c r="AY4" t="s">
         <v>21</v>
       </c>
-      <c r="AZ4" s="1">
+      <c r="AZ4" s="2">
         <v>45555</v>
       </c>
       <c r="BA4" t="s">
@@ -7672,7 +7698,7 @@
       <c r="AY5" t="s">
         <v>21</v>
       </c>
-      <c r="AZ5" s="1">
+      <c r="AZ5" s="2">
         <v>45555</v>
       </c>
       <c r="BA5" t="s">
@@ -7791,7 +7817,7 @@
       <c r="AY6" t="s">
         <v>21</v>
       </c>
-      <c r="AZ6" s="1">
+      <c r="AZ6" s="2">
         <v>45555</v>
       </c>
       <c r="BA6" t="s">
@@ -7910,7 +7936,7 @@
       <c r="AY7" t="s">
         <v>21</v>
       </c>
-      <c r="AZ7" s="1">
+      <c r="AZ7" s="2">
         <v>45555</v>
       </c>
       <c r="BA7" t="s">
@@ -8029,7 +8055,7 @@
       <c r="AY8" t="s">
         <v>21</v>
       </c>
-      <c r="AZ8" s="1">
+      <c r="AZ8" s="2">
         <v>45555</v>
       </c>
       <c r="BA8" t="s">
@@ -8148,7 +8174,7 @@
       <c r="AY9" t="s">
         <v>21</v>
       </c>
-      <c r="AZ9" s="1">
+      <c r="AZ9" s="2">
         <v>45555</v>
       </c>
       <c r="BA9" t="s">
@@ -8258,7 +8284,7 @@
       <c r="AY10" t="s">
         <v>20</v>
       </c>
-      <c r="AZ10" s="1">
+      <c r="AZ10" s="2">
         <v>45835</v>
       </c>
       <c r="BA10" t="s">
@@ -8377,7 +8403,7 @@
       <c r="AY11" t="s">
         <v>21</v>
       </c>
-      <c r="AZ11" s="1">
+      <c r="AZ11" s="2">
         <v>45835</v>
       </c>
       <c r="BA11" t="s">
@@ -8496,7 +8522,7 @@
       <c r="AY12" t="s">
         <v>21</v>
       </c>
-      <c r="AZ12" s="1">
+      <c r="AZ12" s="2">
         <v>45835</v>
       </c>
       <c r="BA12" t="s">
@@ -8615,7 +8641,7 @@
       <c r="AY13" t="s">
         <v>21</v>
       </c>
-      <c r="AZ13" s="1">
+      <c r="AZ13" s="2">
         <v>45835</v>
       </c>
       <c r="BA13" t="s">
@@ -8734,7 +8760,7 @@
       <c r="AY14" t="s">
         <v>21</v>
       </c>
-      <c r="AZ14" s="1">
+      <c r="AZ14" s="2">
         <v>45835</v>
       </c>
       <c r="BA14" t="s">
@@ -8853,7 +8879,7 @@
       <c r="AY15" t="s">
         <v>21</v>
       </c>
-      <c r="AZ15" s="1">
+      <c r="AZ15" s="2">
         <v>45835</v>
       </c>
       <c r="BA15" t="s">
@@ -8972,7 +8998,7 @@
       <c r="AY16" t="s">
         <v>21</v>
       </c>
-      <c r="AZ16" s="1">
+      <c r="AZ16" s="2">
         <v>45835</v>
       </c>
       <c r="BA16" t="s">
@@ -9091,7 +9117,7 @@
       <c r="AY17" t="s">
         <v>21</v>
       </c>
-      <c r="AZ17" s="1">
+      <c r="AZ17" s="2">
         <v>45835</v>
       </c>
       <c r="BA17" t="s">
@@ -9201,7 +9227,7 @@
       <c r="AY18" t="s">
         <v>20</v>
       </c>
-      <c r="AZ18" s="1">
+      <c r="AZ18" s="2">
         <v>45842</v>
       </c>
       <c r="BA18" t="s">
@@ -9323,7 +9349,7 @@
       <c r="AY19" t="s">
         <v>21</v>
       </c>
-      <c r="AZ19" s="1">
+      <c r="AZ19" s="2">
         <v>45842</v>
       </c>
       <c r="BA19" t="s">
@@ -9442,7 +9468,7 @@
       <c r="AY20" t="s">
         <v>21</v>
       </c>
-      <c r="AZ20" s="1">
+      <c r="AZ20" s="2">
         <v>45842</v>
       </c>
       <c r="BA20" t="s">
@@ -9564,7 +9590,7 @@
       <c r="AY21" t="s">
         <v>21</v>
       </c>
-      <c r="AZ21" s="1">
+      <c r="AZ21" s="2">
         <v>45842</v>
       </c>
       <c r="BA21" t="s">
@@ -9686,7 +9712,7 @@
       <c r="AY22" t="s">
         <v>21</v>
       </c>
-      <c r="AZ22" s="1">
+      <c r="AZ22" s="2">
         <v>45842</v>
       </c>
       <c r="BA22" t="s">
@@ -9805,7 +9831,7 @@
       <c r="AY23" t="s">
         <v>21</v>
       </c>
-      <c r="AZ23" s="1">
+      <c r="AZ23" s="2">
         <v>45842</v>
       </c>
       <c r="BA23" t="s">
@@ -9924,7 +9950,7 @@
       <c r="AY24" t="s">
         <v>21</v>
       </c>
-      <c r="AZ24" s="1">
+      <c r="AZ24" s="2">
         <v>45842</v>
       </c>
       <c r="BA24" t="s">
@@ -10043,7 +10069,7 @@
       <c r="AY25" t="s">
         <v>21</v>
       </c>
-      <c r="AZ25" s="1">
+      <c r="AZ25" s="2">
         <v>45842</v>
       </c>
       <c r="BA25" t="s">
@@ -10156,7 +10182,7 @@
       <c r="AY26" t="s">
         <v>20</v>
       </c>
-      <c r="AZ26" s="1">
+      <c r="AZ26" s="2">
         <v>45849</v>
       </c>
       <c r="BA26" t="s">
@@ -10278,7 +10304,7 @@
       <c r="AY27" t="s">
         <v>21</v>
       </c>
-      <c r="AZ27" s="1">
+      <c r="AZ27" s="2">
         <v>45849</v>
       </c>
       <c r="BA27" t="s">
@@ -10400,7 +10426,7 @@
       <c r="AY28" t="s">
         <v>21</v>
       </c>
-      <c r="AZ28" s="1">
+      <c r="AZ28" s="2">
         <v>45849</v>
       </c>
       <c r="BA28" t="s">
@@ -10522,7 +10548,7 @@
       <c r="AY29" t="s">
         <v>21</v>
       </c>
-      <c r="AZ29" s="1">
+      <c r="AZ29" s="2">
         <v>45849</v>
       </c>
       <c r="BA29" t="s">
@@ -10644,7 +10670,7 @@
       <c r="AY30" t="s">
         <v>21</v>
       </c>
-      <c r="AZ30" s="1">
+      <c r="AZ30" s="2">
         <v>45849</v>
       </c>
       <c r="BA30" t="s">
@@ -10763,7 +10789,7 @@
       <c r="AY31" t="s">
         <v>21</v>
       </c>
-      <c r="AZ31" s="1">
+      <c r="AZ31" s="2">
         <v>45849</v>
       </c>
       <c r="BA31" t="s">
@@ -10882,7 +10908,7 @@
       <c r="AY32" t="s">
         <v>21</v>
       </c>
-      <c r="AZ32" s="1">
+      <c r="AZ32" s="2">
         <v>45849</v>
       </c>
       <c r="BA32" t="s">
@@ -11004,7 +11030,7 @@
       <c r="AY33" t="s">
         <v>21</v>
       </c>
-      <c r="AZ33" s="1">
+      <c r="AZ33" s="2">
         <v>45849</v>
       </c>
       <c r="BA33" t="s">
@@ -11117,7 +11143,7 @@
       <c r="AY34" t="s">
         <v>20</v>
       </c>
-      <c r="AZ34" s="1">
+      <c r="AZ34" s="2">
         <v>45856</v>
       </c>
       <c r="BA34" t="s">
@@ -11239,7 +11265,7 @@
       <c r="AY35" t="s">
         <v>21</v>
       </c>
-      <c r="AZ35" s="1">
+      <c r="AZ35" s="2">
         <v>45856</v>
       </c>
       <c r="BA35" t="s">
@@ -11361,7 +11387,7 @@
       <c r="AY36" t="s">
         <v>21</v>
       </c>
-      <c r="AZ36" s="1">
+      <c r="AZ36" s="2">
         <v>45856</v>
       </c>
       <c r="BA36" t="s">
@@ -11483,7 +11509,7 @@
       <c r="AY37" t="s">
         <v>21</v>
       </c>
-      <c r="AZ37" s="1">
+      <c r="AZ37" s="2">
         <v>45856</v>
       </c>
       <c r="BA37" t="s">
@@ -11605,7 +11631,7 @@
       <c r="AY38" t="s">
         <v>21</v>
       </c>
-      <c r="AZ38" s="1">
+      <c r="AZ38" s="2">
         <v>45856</v>
       </c>
       <c r="BA38" t="s">
@@ -11727,7 +11753,7 @@
       <c r="AY39" t="s">
         <v>21</v>
       </c>
-      <c r="AZ39" s="1">
+      <c r="AZ39" s="2">
         <v>45856</v>
       </c>
       <c r="BA39" t="s">
@@ -11846,7 +11872,7 @@
       <c r="AY40" t="s">
         <v>21</v>
       </c>
-      <c r="AZ40" s="1">
+      <c r="AZ40" s="2">
         <v>45856</v>
       </c>
       <c r="BA40" t="s">
@@ -11968,7 +11994,7 @@
       <c r="AY41" t="s">
         <v>21</v>
       </c>
-      <c r="AZ41" s="1">
+      <c r="AZ41" s="2">
         <v>45856</v>
       </c>
       <c r="BA41" t="s">
@@ -12081,7 +12107,7 @@
       <c r="AY42" t="s">
         <v>20</v>
       </c>
-      <c r="AZ42" s="1">
+      <c r="AZ42" s="2">
         <v>45863</v>
       </c>
       <c r="BA42" t="s">
@@ -12203,7 +12229,7 @@
       <c r="AY43" t="s">
         <v>21</v>
       </c>
-      <c r="AZ43" s="1">
+      <c r="AZ43" s="2">
         <v>45863</v>
       </c>
       <c r="BA43" t="s">
@@ -12325,7 +12351,7 @@
       <c r="AY44" t="s">
         <v>21</v>
       </c>
-      <c r="AZ44" s="1">
+      <c r="AZ44" s="2">
         <v>45863</v>
       </c>
       <c r="BA44" t="s">
@@ -12447,7 +12473,7 @@
       <c r="AY45" t="s">
         <v>21</v>
       </c>
-      <c r="AZ45" s="1">
+      <c r="AZ45" s="2">
         <v>45863</v>
       </c>
       <c r="BA45" t="s">
@@ -12569,7 +12595,7 @@
       <c r="AY46" t="s">
         <v>21</v>
       </c>
-      <c r="AZ46" s="1">
+      <c r="AZ46" s="2">
         <v>45863</v>
       </c>
       <c r="BA46" t="s">
@@ -12691,7 +12717,7 @@
       <c r="AY47" t="s">
         <v>21</v>
       </c>
-      <c r="AZ47" s="1">
+      <c r="AZ47" s="2">
         <v>45863</v>
       </c>
       <c r="BA47" t="s">
@@ -12810,7 +12836,7 @@
       <c r="AY48" t="s">
         <v>21</v>
       </c>
-      <c r="AZ48" s="1">
+      <c r="AZ48" s="2">
         <v>45863</v>
       </c>
       <c r="BA48" t="s">
@@ -12932,7 +12958,7 @@
       <c r="AY49" t="s">
         <v>21</v>
       </c>
-      <c r="AZ49" s="1">
+      <c r="AZ49" s="2">
         <v>45863</v>
       </c>
       <c r="BA49" t="s">
@@ -13045,7 +13071,7 @@
       <c r="AY50" t="s">
         <v>20</v>
       </c>
-      <c r="AZ50" s="1">
+      <c r="AZ50" s="2">
         <v>45870</v>
       </c>
       <c r="BA50" t="s">
@@ -13167,7 +13193,7 @@
       <c r="AY51" t="s">
         <v>21</v>
       </c>
-      <c r="AZ51" s="1">
+      <c r="AZ51" s="2">
         <v>45870</v>
       </c>
       <c r="BA51" t="s">
@@ -13289,7 +13315,7 @@
       <c r="AY52" t="s">
         <v>21</v>
       </c>
-      <c r="AZ52" s="1">
+      <c r="AZ52" s="2">
         <v>45870</v>
       </c>
       <c r="BA52" t="s">
@@ -13411,7 +13437,7 @@
       <c r="AY53" t="s">
         <v>21</v>
       </c>
-      <c r="AZ53" s="1">
+      <c r="AZ53" s="2">
         <v>45870</v>
       </c>
       <c r="BA53" t="s">
@@ -13533,7 +13559,7 @@
       <c r="AY54" t="s">
         <v>21</v>
       </c>
-      <c r="AZ54" s="1">
+      <c r="AZ54" s="2">
         <v>45870</v>
       </c>
       <c r="BA54" t="s">
@@ -13655,7 +13681,7 @@
       <c r="AY55" t="s">
         <v>21</v>
       </c>
-      <c r="AZ55" s="1">
+      <c r="AZ55" s="2">
         <v>45870</v>
       </c>
       <c r="BA55" t="s">
@@ -13774,7 +13800,7 @@
       <c r="AY56" t="s">
         <v>21</v>
       </c>
-      <c r="AZ56" s="1">
+      <c r="AZ56" s="2">
         <v>45870</v>
       </c>
       <c r="BA56" t="s">
@@ -13896,7 +13922,7 @@
       <c r="AY57" t="s">
         <v>21</v>
       </c>
-      <c r="AZ57" s="1">
+      <c r="AZ57" s="2">
         <v>45870</v>
       </c>
       <c r="BA57" t="s">
@@ -14009,7 +14035,7 @@
       <c r="AY58" t="s">
         <v>20</v>
       </c>
-      <c r="AZ58" s="1">
+      <c r="AZ58" s="2">
         <v>45877</v>
       </c>
       <c r="BA58" t="s">
@@ -14131,7 +14157,7 @@
       <c r="AY59" t="s">
         <v>21</v>
       </c>
-      <c r="AZ59" s="1">
+      <c r="AZ59" s="2">
         <v>45877</v>
       </c>
       <c r="BA59" t="s">
@@ -14253,7 +14279,7 @@
       <c r="AY60" t="s">
         <v>21</v>
       </c>
-      <c r="AZ60" s="1">
+      <c r="AZ60" s="2">
         <v>45877</v>
       </c>
       <c r="BA60" t="s">
@@ -14375,7 +14401,7 @@
       <c r="AY61" t="s">
         <v>21</v>
       </c>
-      <c r="AZ61" s="1">
+      <c r="AZ61" s="2">
         <v>45877</v>
       </c>
       <c r="BA61" t="s">
@@ -14497,7 +14523,7 @@
       <c r="AY62" t="s">
         <v>21</v>
       </c>
-      <c r="AZ62" s="1">
+      <c r="AZ62" s="2">
         <v>45877</v>
       </c>
       <c r="BA62" t="s">
@@ -14619,7 +14645,7 @@
       <c r="AY63" t="s">
         <v>21</v>
       </c>
-      <c r="AZ63" s="1">
+      <c r="AZ63" s="2">
         <v>45877</v>
       </c>
       <c r="BA63" t="s">
@@ -14738,7 +14764,7 @@
       <c r="AY64" t="s">
         <v>21</v>
       </c>
-      <c r="AZ64" s="1">
+      <c r="AZ64" s="2">
         <v>45877</v>
       </c>
       <c r="BA64" t="s">
@@ -14860,7 +14886,7 @@
       <c r="AY65" t="s">
         <v>21</v>
       </c>
-      <c r="AZ65" s="1">
+      <c r="AZ65" s="2">
         <v>45877</v>
       </c>
       <c r="BA65" t="s">
@@ -14973,7 +14999,7 @@
       <c r="AY66" t="s">
         <v>20</v>
       </c>
-      <c r="AZ66" s="1">
+      <c r="AZ66" s="2">
         <v>45884</v>
       </c>
       <c r="BA66" t="s">
@@ -15095,7 +15121,7 @@
       <c r="AY67" t="s">
         <v>21</v>
       </c>
-      <c r="AZ67" s="1">
+      <c r="AZ67" s="2">
         <v>45884</v>
       </c>
       <c r="BA67" t="s">
@@ -15217,7 +15243,7 @@
       <c r="AY68" t="s">
         <v>21</v>
       </c>
-      <c r="AZ68" s="1">
+      <c r="AZ68" s="2">
         <v>45884</v>
       </c>
       <c r="BA68" t="s">
@@ -15339,7 +15365,7 @@
       <c r="AY69" t="s">
         <v>21</v>
       </c>
-      <c r="AZ69" s="1">
+      <c r="AZ69" s="2">
         <v>45884</v>
       </c>
       <c r="BA69" t="s">
@@ -15461,7 +15487,7 @@
       <c r="AY70" t="s">
         <v>21</v>
       </c>
-      <c r="AZ70" s="1">
+      <c r="AZ70" s="2">
         <v>45884</v>
       </c>
       <c r="BA70" t="s">
@@ -15583,7 +15609,7 @@
       <c r="AY71" t="s">
         <v>21</v>
       </c>
-      <c r="AZ71" s="1">
+      <c r="AZ71" s="2">
         <v>45884</v>
       </c>
       <c r="BA71" t="s">
@@ -15702,7 +15728,7 @@
       <c r="AY72" t="s">
         <v>21</v>
       </c>
-      <c r="AZ72" s="1">
+      <c r="AZ72" s="2">
         <v>45884</v>
       </c>
       <c r="BA72" t="s">
@@ -15824,7 +15850,7 @@
       <c r="AY73" t="s">
         <v>21</v>
       </c>
-      <c r="AZ73" s="1">
+      <c r="AZ73" s="2">
         <v>45884</v>
       </c>
       <c r="BA73" t="s">
@@ -15937,7 +15963,7 @@
       <c r="AY74" t="s">
         <v>20</v>
       </c>
-      <c r="AZ74" s="1">
+      <c r="AZ74" s="2">
         <v>45891</v>
       </c>
       <c r="BA74" t="s">
@@ -16059,7 +16085,7 @@
       <c r="AY75" t="s">
         <v>21</v>
       </c>
-      <c r="AZ75" s="1">
+      <c r="AZ75" s="2">
         <v>45891</v>
       </c>
       <c r="BA75" t="s">
@@ -16181,7 +16207,7 @@
       <c r="AY76" t="s">
         <v>21</v>
       </c>
-      <c r="AZ76" s="1">
+      <c r="AZ76" s="2">
         <v>45891</v>
       </c>
       <c r="BA76" t="s">
@@ -16303,7 +16329,7 @@
       <c r="AY77" t="s">
         <v>21</v>
       </c>
-      <c r="AZ77" s="1">
+      <c r="AZ77" s="2">
         <v>45891</v>
       </c>
       <c r="BA77" t="s">
@@ -16425,7 +16451,7 @@
       <c r="AY78" t="s">
         <v>21</v>
       </c>
-      <c r="AZ78" s="1">
+      <c r="AZ78" s="2">
         <v>45891</v>
       </c>
       <c r="BA78" t="s">
@@ -16547,7 +16573,7 @@
       <c r="AY79" t="s">
         <v>21</v>
       </c>
-      <c r="AZ79" s="1">
+      <c r="AZ79" s="2">
         <v>45891</v>
       </c>
       <c r="BA79" t="s">
@@ -16666,7 +16692,7 @@
       <c r="AY80" t="s">
         <v>21</v>
       </c>
-      <c r="AZ80" s="1">
+      <c r="AZ80" s="2">
         <v>45891</v>
       </c>
       <c r="BA80" t="s">
@@ -16788,7 +16814,7 @@
       <c r="AY81" t="s">
         <v>21</v>
       </c>
-      <c r="AZ81" s="1">
+      <c r="AZ81" s="2">
         <v>45891</v>
       </c>
       <c r="BA81" t="s">
@@ -16901,7 +16927,7 @@
       <c r="AY82" t="s">
         <v>20</v>
       </c>
-      <c r="AZ82" s="1">
+      <c r="AZ82" s="2">
         <v>45898</v>
       </c>
       <c r="BA82" t="s">
@@ -17023,7 +17049,7 @@
       <c r="AY83" t="s">
         <v>21</v>
       </c>
-      <c r="AZ83" s="1">
+      <c r="AZ83" s="2">
         <v>45898</v>
       </c>
       <c r="BA83" t="s">
@@ -17145,7 +17171,7 @@
       <c r="AY84" t="s">
         <v>21</v>
       </c>
-      <c r="AZ84" s="1">
+      <c r="AZ84" s="2">
         <v>45898</v>
       </c>
       <c r="BA84" t="s">
@@ -17267,7 +17293,7 @@
       <c r="AY85" t="s">
         <v>21</v>
       </c>
-      <c r="AZ85" s="1">
+      <c r="AZ85" s="2">
         <v>45898</v>
       </c>
       <c r="BA85" t="s">
@@ -17389,7 +17415,7 @@
       <c r="AY86" t="s">
         <v>21</v>
       </c>
-      <c r="AZ86" s="1">
+      <c r="AZ86" s="2">
         <v>45898</v>
       </c>
       <c r="BA86" t="s">
@@ -17511,7 +17537,7 @@
       <c r="AY87" t="s">
         <v>21</v>
       </c>
-      <c r="AZ87" s="1">
+      <c r="AZ87" s="2">
         <v>45898</v>
       </c>
       <c r="BA87" t="s">
@@ -17630,7 +17656,7 @@
       <c r="AY88" t="s">
         <v>21</v>
       </c>
-      <c r="AZ88" s="1">
+      <c r="AZ88" s="2">
         <v>45898</v>
       </c>
       <c r="BA88" t="s">
@@ -17752,7 +17778,7 @@
       <c r="AY89" t="s">
         <v>21</v>
       </c>
-      <c r="AZ89" s="1">
+      <c r="AZ89" s="2">
         <v>45898</v>
       </c>
       <c r="BA89" t="s">
@@ -17865,7 +17891,7 @@
       <c r="AY90" t="s">
         <v>20</v>
       </c>
-      <c r="AZ90" s="1">
+      <c r="AZ90" s="2">
         <v>45905</v>
       </c>
       <c r="BA90" t="s">
@@ -17987,7 +18013,7 @@
       <c r="AY91" t="s">
         <v>21</v>
       </c>
-      <c r="AZ91" s="1">
+      <c r="AZ91" s="2">
         <v>45905</v>
       </c>
       <c r="BA91" t="s">
@@ -18109,7 +18135,7 @@
       <c r="AY92" t="s">
         <v>21</v>
       </c>
-      <c r="AZ92" s="1">
+      <c r="AZ92" s="2">
         <v>45905</v>
       </c>
       <c r="BA92" t="s">
@@ -18231,7 +18257,7 @@
       <c r="AY93" t="s">
         <v>21</v>
       </c>
-      <c r="AZ93" s="1">
+      <c r="AZ93" s="2">
         <v>45905</v>
       </c>
       <c r="BA93" t="s">
@@ -18353,7 +18379,7 @@
       <c r="AY94" t="s">
         <v>21</v>
       </c>
-      <c r="AZ94" s="1">
+      <c r="AZ94" s="2">
         <v>45905</v>
       </c>
       <c r="BA94" t="s">
@@ -18475,7 +18501,7 @@
       <c r="AY95" t="s">
         <v>21</v>
       </c>
-      <c r="AZ95" s="1">
+      <c r="AZ95" s="2">
         <v>45905</v>
       </c>
       <c r="BA95" t="s">
@@ -18594,7 +18620,7 @@
       <c r="AY96" t="s">
         <v>21</v>
       </c>
-      <c r="AZ96" s="1">
+      <c r="AZ96" s="2">
         <v>45905</v>
       </c>
       <c r="BA96" t="s">
@@ -18716,7 +18742,7 @@
       <c r="AY97" t="s">
         <v>21</v>
       </c>
-      <c r="AZ97" s="1">
+      <c r="AZ97" s="2">
         <v>45905</v>
       </c>
       <c r="BA97" t="s">
@@ -18829,7 +18855,7 @@
       <c r="AY98" t="s">
         <v>20</v>
       </c>
-      <c r="AZ98" s="1">
+      <c r="AZ98" s="2">
         <v>45912</v>
       </c>
       <c r="BA98" t="s">
@@ -18951,7 +18977,7 @@
       <c r="AY99" t="s">
         <v>21</v>
       </c>
-      <c r="AZ99" s="1">
+      <c r="AZ99" s="2">
         <v>45912</v>
       </c>
       <c r="BA99" t="s">
@@ -19073,7 +19099,7 @@
       <c r="AY100" t="s">
         <v>21</v>
       </c>
-      <c r="AZ100" s="1">
+      <c r="AZ100" s="2">
         <v>45912</v>
       </c>
       <c r="BA100" t="s">
@@ -19195,7 +19221,7 @@
       <c r="AY101" t="s">
         <v>21</v>
       </c>
-      <c r="AZ101" s="1">
+      <c r="AZ101" s="2">
         <v>45912</v>
       </c>
       <c r="BA101" t="s">
@@ -19317,7 +19343,7 @@
       <c r="AY102" t="s">
         <v>21</v>
       </c>
-      <c r="AZ102" s="1">
+      <c r="AZ102" s="2">
         <v>45912</v>
       </c>
       <c r="BA102" t="s">
@@ -19439,7 +19465,7 @@
       <c r="AY103" t="s">
         <v>21</v>
       </c>
-      <c r="AZ103" s="1">
+      <c r="AZ103" s="2">
         <v>45912</v>
       </c>
       <c r="BA103" t="s">
@@ -19558,7 +19584,7 @@
       <c r="AY104" t="s">
         <v>21</v>
       </c>
-      <c r="AZ104" s="1">
+      <c r="AZ104" s="2">
         <v>45912</v>
       </c>
       <c r="BA104" t="s">
@@ -19680,7 +19706,7 @@
       <c r="AY105" t="s">
         <v>21</v>
       </c>
-      <c r="AZ105" s="1">
+      <c r="AZ105" s="2">
         <v>45912</v>
       </c>
       <c r="BA105" t="s">
@@ -19793,7 +19819,7 @@
       <c r="AY106" t="s">
         <v>20</v>
       </c>
-      <c r="AZ106" s="1">
+      <c r="AZ106" s="2">
         <v>45919</v>
       </c>
       <c r="BA106" t="s">
@@ -19915,7 +19941,7 @@
       <c r="AY107" t="s">
         <v>21</v>
       </c>
-      <c r="AZ107" s="1">
+      <c r="AZ107" s="2">
         <v>45919</v>
       </c>
       <c r="BA107" t="s">
@@ -20037,7 +20063,7 @@
       <c r="AY108" t="s">
         <v>21</v>
       </c>
-      <c r="AZ108" s="1">
+      <c r="AZ108" s="2">
         <v>45919</v>
       </c>
       <c r="BA108" t="s">
@@ -20159,7 +20185,7 @@
       <c r="AY109" t="s">
         <v>21</v>
       </c>
-      <c r="AZ109" s="1">
+      <c r="AZ109" s="2">
         <v>45919</v>
       </c>
       <c r="BA109" t="s">
@@ -20281,7 +20307,7 @@
       <c r="AY110" t="s">
         <v>21</v>
       </c>
-      <c r="AZ110" s="1">
+      <c r="AZ110" s="2">
         <v>45919</v>
       </c>
       <c r="BA110" t="s">
@@ -20403,7 +20429,7 @@
       <c r="AY111" t="s">
         <v>21</v>
       </c>
-      <c r="AZ111" s="1">
+      <c r="AZ111" s="2">
         <v>45919</v>
       </c>
       <c r="BA111" t="s">
@@ -20522,7 +20548,7 @@
       <c r="AY112" t="s">
         <v>21</v>
       </c>
-      <c r="AZ112" s="1">
+      <c r="AZ112" s="2">
         <v>45919</v>
       </c>
       <c r="BA112" t="s">
@@ -20644,7 +20670,7 @@
       <c r="AY113" t="s">
         <v>21</v>
       </c>
-      <c r="AZ113" s="1">
+      <c r="AZ113" s="2">
         <v>45919</v>
       </c>
       <c r="BA113" t="s">
@@ -20757,7 +20783,7 @@
       <c r="AY114" t="s">
         <v>20</v>
       </c>
-      <c r="AZ114" s="1">
+      <c r="AZ114" s="2">
         <v>45926</v>
       </c>
       <c r="BA114" t="s">
@@ -20879,7 +20905,7 @@
       <c r="AY115" t="s">
         <v>21</v>
       </c>
-      <c r="AZ115" s="1">
+      <c r="AZ115" s="2">
         <v>45926</v>
       </c>
       <c r="BA115" t="s">
@@ -21001,7 +21027,7 @@
       <c r="AY116" t="s">
         <v>21</v>
       </c>
-      <c r="AZ116" s="1">
+      <c r="AZ116" s="2">
         <v>45926</v>
       </c>
       <c r="BA116" t="s">
@@ -21123,7 +21149,7 @@
       <c r="AY117" t="s">
         <v>21</v>
       </c>
-      <c r="AZ117" s="1">
+      <c r="AZ117" s="2">
         <v>45926</v>
       </c>
       <c r="BA117" t="s">
@@ -21245,7 +21271,7 @@
       <c r="AY118" t="s">
         <v>21</v>
       </c>
-      <c r="AZ118" s="1">
+      <c r="AZ118" s="2">
         <v>45926</v>
       </c>
       <c r="BA118" t="s">
@@ -21367,7 +21393,7 @@
       <c r="AY119" t="s">
         <v>21</v>
       </c>
-      <c r="AZ119" s="1">
+      <c r="AZ119" s="2">
         <v>45926</v>
       </c>
       <c r="BA119" t="s">
@@ -21486,7 +21512,7 @@
       <c r="AY120" t="s">
         <v>21</v>
       </c>
-      <c r="AZ120" s="1">
+      <c r="AZ120" s="2">
         <v>45926</v>
       </c>
       <c r="BA120" t="s">
@@ -21608,7 +21634,7 @@
       <c r="AY121" t="s">
         <v>21</v>
       </c>
-      <c r="AZ121" s="1">
+      <c r="AZ121" s="2">
         <v>45926</v>
       </c>
       <c r="BA121" t="s">

</xml_diff>